<commit_message>
Corrida | ARG-MVDO | 2026-09-04 09:54:11.873478
</commit_message>
<xml_diff>
--- a/indicadores/ARG-MVDO_out.xlsx
+++ b/indicadores/ARG-MVDO_out.xlsx
@@ -110,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">03/09/2026</t>
+    <t xml:space="preserve">04/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2187,7 +2187,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.51162496256058</v>
+        <v>0.510449160594468</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2245,7 +2245,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.186777346040514</v>
+        <v>0.186491162385076</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2315,7 +2315,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000359541294965735</v>
+        <v>0.000379160166214667</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2345,7 +2345,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.809274552855928</v>
+        <v>0.820723333694641</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -27126,7 +27126,7 @@
         <v>518</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.226458123407064</v>
+        <v>0.226931414062566</v>
       </c>
     </row>
     <row r="6">
@@ -27134,7 +27134,7 @@
         <v>519</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.237685389135388</v>
+        <v>0.238178720466985</v>
       </c>
     </row>
     <row r="7">
@@ -27142,7 +27142,7 @@
         <v>520</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.264115186725624</v>
+        <v>0.263474507602288</v>
       </c>
     </row>
     <row r="8">
@@ -27150,7 +27150,7 @@
         <v>521</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.309979208478606</v>
+        <v>0.307305394616396</v>
       </c>
     </row>
     <row r="9">
@@ -27158,7 +27158,7 @@
         <v>522</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.364118841622459</v>
+        <v>0.361848233232408</v>
       </c>
     </row>
     <row r="10">
@@ -27166,7 +27166,7 @@
         <v>523</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.424214286018579</v>
+        <v>0.423279455936072</v>
       </c>
     </row>
     <row r="11">
@@ -27174,7 +27174,7 @@
         <v>524</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.475169601969946</v>
+        <v>0.473642567093454</v>
       </c>
     </row>
     <row r="12">
@@ -27182,7 +27182,7 @@
         <v>525</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.51162496256058</v>
+        <v>0.510449160594468</v>
       </c>
     </row>
     <row r="13">
@@ -27190,7 +27190,7 @@
         <v>526</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.50264535536231</v>
+        <v>0.503060907639816</v>
       </c>
     </row>
     <row r="14">
@@ -27198,7 +27198,7 @@
         <v>527</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.432177447399229</v>
+        <v>0.431846225391719</v>
       </c>
     </row>
     <row r="15">
@@ -27206,7 +27206,7 @@
         <v>528</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.329372883852987</v>
+        <v>0.3290182817672</v>
       </c>
     </row>
     <row r="16">
@@ -27214,7 +27214,7 @@
         <v>529</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.231037595075791</v>
+        <v>0.233480621763414</v>
       </c>
     </row>
     <row r="17">
@@ -27222,7 +27222,7 @@
         <v>530</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.16451343468717</v>
+        <v>0.168332670603179</v>
       </c>
     </row>
     <row r="18">
@@ -27230,7 +27230,7 @@
         <v>531</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.13041503928118</v>
+        <v>0.132161478515735</v>
       </c>
     </row>
     <row r="19">
@@ -27238,7 +27238,7 @@
         <v>532</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.103093352668006</v>
+        <v>0.101522446785895</v>
       </c>
     </row>
     <row r="20">
@@ -27246,7 +27246,7 @@
         <v>533</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0537566232551183</v>
+        <v>0.0516503084572329</v>
       </c>
     </row>
     <row r="21">
@@ -27254,7 +27254,7 @@
         <v>534</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.00331901588452541</v>
+        <v>-0.00317013967360938</v>
       </c>
     </row>
     <row r="22">
@@ -27262,7 +27262,7 @@
         <v>535</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0525041731789284</v>
+        <v>-0.05035864878914</v>
       </c>
     </row>
     <row r="23">
@@ -27270,7 +27270,7 @@
         <v>536</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0890194857221719</v>
+        <v>-0.0860827850620026</v>
       </c>
     </row>
     <row r="24">

</xml_diff>